<commit_message>
added the data for day 2
</commit_message>
<xml_diff>
--- a/12618117.xlsx
+++ b/12618117.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krish\Desktop\MCA_SEM1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FBE4676-770F-4FCD-A18F-306E2D7B1D26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9FBD5B-EF3C-47CF-B375-5E9983653D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -203,6 +203,15 @@
   </si>
   <si>
     <t>Extreme humidity</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Satisfied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today I explained a code infront of the class. </t>
   </si>
 </sst>
 </file>
@@ -983,7 +992,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
-        <v>46223</v>
+        <v>46246</v>
       </c>
       <c r="B6" s="9">
         <v>480</v>
@@ -1027,27 +1036,51 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15" t="str">
+    <row r="7" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="8">
+        <v>46247</v>
+      </c>
+      <c r="B7" s="14">
+        <v>380</v>
+      </c>
+      <c r="C7" s="14">
+        <v>30</v>
+      </c>
+      <c r="D7" s="14">
+        <v>60</v>
+      </c>
+      <c r="E7" s="14">
+        <v>60</v>
+      </c>
+      <c r="F7" s="14">
+        <v>480</v>
+      </c>
+      <c r="G7" s="14">
+        <v>8</v>
+      </c>
+      <c r="H7" s="14">
+        <v>150</v>
+      </c>
+      <c r="I7" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="15" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="17"/>
+        <v>280</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="13"/>

</xml_diff>

<commit_message>
added the data for day 3
</commit_message>
<xml_diff>
--- a/12618117.xlsx
+++ b/12618117.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krish\Desktop\MCA_SEM1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F879FBE-C4AC-4338-88DF-8950005BC27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E125653-AD3C-4424-BB0F-04155F80C4A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -218,6 +218,12 @@
   </si>
   <si>
     <t xml:space="preserve">It was a good day. </t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>It was holiday and the day didn't had much activity.</t>
   </si>
 </sst>
 </file>
@@ -1134,27 +1140,51 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+    <row r="9" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="8">
+        <v>46249</v>
+      </c>
+      <c r="B9" s="14">
+        <v>360</v>
+      </c>
+      <c r="C9" s="14">
+        <v>15</v>
+      </c>
+      <c r="D9" s="14">
+        <v>45</v>
+      </c>
+      <c r="E9" s="14">
+        <v>30</v>
+      </c>
+      <c r="F9" s="14">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14">
+        <v>440</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>550</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>

</xml_diff>